<commit_message>
exec review: discount-leakage drill-down slide; rebuild deliverables
New slide 7 (waterfall gross -> within-policy -> excess -> net, top-6 reps
by excess-over-policy, top-offender callout); PDF/PPTX now 9 slides.
Deliverables regenerated with the drill-down in analysis.json, QBR
markdown, workbook and the new leakage_waterfall.png.
</commit_message>
<xml_diff>
--- a/deliverables/kpi_workbook.xlsx
+++ b/deliverables/kpi_workbook.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecasts" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reorder list" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spend" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leakage drill-down" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3149,4 +3150,653 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>sales_rep</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>leakage_eur</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>excess_eur</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>within_policy_eur</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>leakage_pct_of_revenue</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>orders</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>orders_above_policy_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>median_discount_pct</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>p90_discount_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Berg</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nordics</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>268809.88</v>
+      </c>
+      <c r="D2" t="n">
+        <v>75779.12</v>
+      </c>
+      <c r="E2" t="n">
+        <v>193030.77</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1256</v>
+      </c>
+      <c r="H2" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J2" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nowak</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>292291.68</v>
+      </c>
+      <c r="D3" t="n">
+        <v>73367.53999999999</v>
+      </c>
+      <c r="E3" t="n">
+        <v>218924.14</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1705</v>
+      </c>
+      <c r="H3" t="n">
+        <v>28.68</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>255726.32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>67365.46000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>188360.86</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1319</v>
+      </c>
+      <c r="H4" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J4" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Braun</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DACH-North</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>193020.03</v>
+      </c>
+      <c r="D5" t="n">
+        <v>61165.41</v>
+      </c>
+      <c r="E5" t="n">
+        <v>131854.61</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1005</v>
+      </c>
+      <c r="H5" t="n">
+        <v>38.11</v>
+      </c>
+      <c r="I5" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="J5" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lindqvist</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nordics</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>227292.66</v>
+      </c>
+      <c r="D6" t="n">
+        <v>58971.41</v>
+      </c>
+      <c r="E6" t="n">
+        <v>168321.26</v>
+      </c>
+      <c r="F6" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1320</v>
+      </c>
+      <c r="H6" t="n">
+        <v>33.86</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="J6" t="n">
+        <v>15.41</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Huber</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DACH-South</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>226439.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>57778.63</v>
+      </c>
+      <c r="E7" t="n">
+        <v>168660.57</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1238</v>
+      </c>
+      <c r="H7" t="n">
+        <v>29.81</v>
+      </c>
+      <c r="I7" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kovac</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>230501.81</v>
+      </c>
+      <c r="D8" t="n">
+        <v>56835.43</v>
+      </c>
+      <c r="E8" t="n">
+        <v>173666.39</v>
+      </c>
+      <c r="F8" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1618</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31.95</v>
+      </c>
+      <c r="I8" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="J8" t="n">
+        <v>14.93</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fischer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DACH-South</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>211609.99</v>
+      </c>
+      <c r="D9" t="n">
+        <v>56449.13</v>
+      </c>
+      <c r="E9" t="n">
+        <v>155160.86</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1211</v>
+      </c>
+      <c r="H9" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dubois</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>209606.69</v>
+      </c>
+      <c r="D10" t="n">
+        <v>50626.49</v>
+      </c>
+      <c r="E10" t="n">
+        <v>158980.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1260</v>
+      </c>
+      <c r="H10" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Weber</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DACH-North</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>183968.93</v>
+      </c>
+      <c r="D11" t="n">
+        <v>47920.45</v>
+      </c>
+      <c r="E11" t="n">
+        <v>136048.49</v>
+      </c>
+      <c r="F11" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1031</v>
+      </c>
+      <c r="H11" t="n">
+        <v>37.54</v>
+      </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mayer</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DACH-South</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>177868.8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>40980.51</v>
+      </c>
+      <c r="E12" t="n">
+        <v>136888.29</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1282</v>
+      </c>
+      <c r="H12" t="n">
+        <v>28.86</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J12" t="n">
+        <v>14.89</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Klein</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DACH-North</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>137766.64</v>
+      </c>
+      <c r="D13" t="n">
+        <v>33485.41</v>
+      </c>
+      <c r="E13" t="n">
+        <v>104281.23</v>
+      </c>
+      <c r="F13" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="G13" t="n">
+        <v>972</v>
+      </c>
+      <c r="H13" t="n">
+        <v>32</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>By region</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>leakage_eur</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>excess_eur</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>leakage_pct_of_revenue</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>orders_above_policy_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DACH-South</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>615917.99</v>
+      </c>
+      <c r="C17" t="n">
+        <v>155208.28</v>
+      </c>
+      <c r="D17" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="E17" t="n">
+        <v>29.54</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DACH-North</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>514755.59</v>
+      </c>
+      <c r="C18" t="n">
+        <v>142571.27</v>
+      </c>
+      <c r="D18" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="E18" t="n">
+        <v>35.94</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nordics</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>496102.54</v>
+      </c>
+      <c r="C19" t="n">
+        <v>134750.52</v>
+      </c>
+      <c r="D19" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="E19" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>522793.49</v>
+      </c>
+      <c r="C20" t="n">
+        <v>130202.97</v>
+      </c>
+      <c r="D20" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="E20" t="n">
+        <v>30.27</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>465333</v>
+      </c>
+      <c r="C21" t="n">
+        <v>117991.95</v>
+      </c>
+      <c r="D21" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="E21" t="n">
+        <v>32.57</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Policy threshold %</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>assumed sanctioned-discount ceiling (no contract terms in the dataset); within-policy vs excess split depends on it, the total leakage does not</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>